<commit_message>
fix(evaluation): auditoria e correcao cientifica da avaliacao de deteccao de objetos com IoU 0.45 e background
</commit_message>
<xml_diff>
--- a/reports/metricas_mestrado.xlsx
+++ b/reports/metricas_mestrado.xlsx
@@ -70,7 +70,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -87,12 +87,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.0000</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -104,12 +104,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.0000</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -121,12 +121,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1.0000</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -138,12 +138,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1.0000</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -155,12 +155,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1.0000</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -172,12 +172,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1.0000</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -189,12 +189,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1.0000</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -206,12 +206,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1.0000</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -223,12 +223,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0.3573</t>
+          <t>0.9890</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>35.73%</t>
+          <t>98.90%</t>
         </is>
       </c>
     </row>
@@ -240,12 +240,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0.2748</t>
+          <t>0.7211</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>27.48%</t>
+          <t>72.11%</t>
         </is>
       </c>
     </row>
@@ -257,7 +257,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>82.82</t>
+          <t>75.82</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -274,7 +274,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>13.2</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -347,120 +347,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>hotspot group</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>57</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>57</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>panel with hotspots</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>57</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>1.0000</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>